<commit_message>
merge ndvi mean to master dataset monthly
</commit_message>
<xml_diff>
--- a/basins/ndvi_per_river.xlsx
+++ b/basins/ndvi_per_river.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2cdde6c514a5c013/Maastricht Study/Semester 1/Research Project S2/Lake Tanganyika/Lake-Tanganyika/basins/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{CD10621E-A1A7-5F4C-A3B0-E34AE003F5F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C815E51-A193-3547-9390-3547E4E8E02E}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="8_{CD10621E-A1A7-5F4C-A3B0-E34AE003F5F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6090AE0-C714-E14D-AD2B-4B7430DBC02C}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="660" windowWidth="28040" windowHeight="16840" xr2:uid="{9C391A78-198C-F245-BEE6-D661AA3F5A64}"/>
+    <workbookView xWindow="680" yWindow="660" windowWidth="28040" windowHeight="16740" xr2:uid="{9C391A78-198C-F245-BEE6-D661AA3F5A64}"/>
   </bookViews>
   <sheets>
     <sheet name="ndvi_per_river" sheetId="1" r:id="rId1"/>
@@ -11967,7 +11967,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="m/d/yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="m/d/yyyy;@"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
@@ -12454,7 +12454,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -12513,6 +12513,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>